<commit_message>
Make the starter pane visible to Excel and skip a missing preview.
Excel for Mac reads taskpanes.xml from the package relationships, so both starter workbooks now point at that part from _rels/.rels. A linked cell whose file is gone names that file and stays in the task pane. Reopening a workbook writes settings only when they changed.

Co-authored-by: jarvis-pd21 <jarvis-pd21@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/datasniper/DataSniper-Starter-alt.xlsx
+++ b/datasniper/DataSniper-Starter-alt.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24106"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet name="DataSniper" sheetId="1" r:id="rId1"/>
+    <sheet name="Start here" sheetId="2" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -38,9 +42,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -71,16 +76,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="96" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DataSniper starter. This workbook opens with the task pane visible. Save it after you snip, and Excel for Mac keeps the pane with the file.</t>
+          <t>DataSniper is ready. This workbook opens with the task pane visible, and Excel for Mac keeps it visible when you save. Export onto the DataSniper sheet so this note stays put.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make the starter pane visible to Excel and skip a missing preview. (#16)
Excel for Mac reads taskpanes.xml from the package relationships, so both starter workbooks now point at that part from _rels/.rels. A linked cell whose file is gone names that file and stays in the task pane. Reopening a workbook writes settings only when they changed.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: jarvis-pd21 <jarvis-pd21@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/datasniper/DataSniper-Starter-alt.xlsx
+++ b/datasniper/DataSniper-Starter-alt.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24106"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet name="DataSniper" sheetId="1" r:id="rId1"/>
+    <sheet name="Start here" sheetId="2" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -38,9 +42,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -71,16 +76,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="96" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DataSniper starter. This workbook opens with the task pane visible. Save it after you snip, and Excel for Mac keeps the pane with the file.</t>
+          <t>DataSniper is ready. This workbook opens with the task pane visible, and Excel for Mac keeps it visible when you save. Export onto the DataSniper sheet so this note stays put.</t>
         </is>
       </c>
     </row>

</xml_diff>